<commit_message>
Bulk filing: keep only three warnings
Bulk scrutiny now raises only these warnings:
- cheque presented after its three-month validity (CHQ-11)
- a scan too blurry or cropped to read (new to bulk; same readability check as the
  single filing, shown on the Documents tab with Replace / Keep this file)
- past the one-month limit with no condonation reason (JUR-12)

Removed: the "not insufficient funds" return-reason warning (other return reasons
still attract S-138) and the late-notice warning. Single filing is unchanged.

Sample spreadsheet: TCL-AHD-PL-1002 is presented late, TCL-AHD-PL-1004 is past the
limit; "Fill with demo files" puts a blurry scan on the first case.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/apps/dristi-app/public/samples/tata-capital-recovery-mis.xlsx
+++ b/apps/dristi-app/public/samples/tata-capital-recovery-mis.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="339" uniqueCount="203">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="339" uniqueCount="206">
   <si>
     <t>Sr No</t>
   </si>
@@ -154,253 +154,397 @@
     <t>38291004512</t>
   </si>
   <si>
+    <t>19/09/2026</t>
+  </si>
+  <si>
+    <t>INSUFFICIENT FUNDS</t>
+  </si>
+  <si>
+    <t>HDFC0000060</t>
+  </si>
+  <si>
+    <t>25/09/2026</t>
+  </si>
+  <si>
+    <t>Regd. Post A/D</t>
+  </si>
+  <si>
+    <t>RG20451111IN</t>
+  </si>
+  <si>
+    <t>SERVED</t>
+  </si>
+  <si>
+    <t>03/10/2026</t>
+  </si>
+  <si>
+    <t>N</t>
+  </si>
+  <si>
+    <t>TCL-AHD-PL-1002</t>
+  </si>
+  <si>
+    <t>Snehal K. Mistry</t>
+  </si>
+  <si>
+    <t>+91 98790 12302</t>
+  </si>
+  <si>
+    <t>snehal.mistry@mail.example</t>
+  </si>
+  <si>
+    <t>14, Gokul Row Houses, Naranpura</t>
+  </si>
+  <si>
+    <t>380013</t>
+  </si>
+  <si>
+    <t>331207</t>
+  </si>
+  <si>
+    <t>92,750</t>
+  </si>
+  <si>
+    <t>HDFC0000521</t>
+  </si>
+  <si>
+    <t>50100221834</t>
+  </si>
+  <si>
     <t>18/09/2026</t>
   </si>
   <si>
-    <t>INSUFFICIENT FUNDS</t>
-  </si>
-  <si>
-    <t>HDFC0000060</t>
-  </si>
-  <si>
     <t>24/09/2026</t>
   </si>
   <si>
-    <t>Regd. Post A/D</t>
-  </si>
-  <si>
-    <t>RG20451111IN</t>
-  </si>
-  <si>
-    <t>SERVED</t>
+    <t>RG33120711IN</t>
   </si>
   <si>
     <t>02/10/2026</t>
   </si>
   <si>
-    <t>N</t>
-  </si>
-  <si>
-    <t>TCL-AHD-PL-1002</t>
-  </si>
-  <si>
-    <t>Snehal K. Mistry</t>
-  </si>
-  <si>
-    <t>+91 98790 12302</t>
-  </si>
-  <si>
-    <t>snehal.mistry@mail.example</t>
-  </si>
-  <si>
-    <t>14, Gokul Row Houses, Naranpura</t>
-  </si>
-  <si>
-    <t>380013</t>
-  </si>
-  <si>
-    <t>331207</t>
-  </si>
-  <si>
-    <t>92,750</t>
-  </si>
-  <si>
-    <t>HDFC0000521</t>
-  </si>
-  <si>
-    <t>50100221834</t>
+    <t>TCL-AHD-BL-1003</t>
+  </si>
+  <si>
+    <t>Business Loan</t>
+  </si>
+  <si>
+    <t>Pravin D. Solanki</t>
+  </si>
+  <si>
+    <t>+91 98790 12303</t>
+  </si>
+  <si>
+    <t>pravin.solanki@mail.example</t>
+  </si>
+  <si>
+    <t>7, Shreeji Society, Maninagar</t>
+  </si>
+  <si>
+    <t>380008</t>
+  </si>
+  <si>
+    <t>118034</t>
+  </si>
+  <si>
+    <t>3,65,000</t>
+  </si>
+  <si>
+    <t>BARB0MANINA</t>
+  </si>
+  <si>
+    <t>21950100004471</t>
   </si>
   <si>
     <t>17/09/2026</t>
   </si>
   <si>
+    <t>EXCEEDS ARRANGEMENT</t>
+  </si>
+  <si>
     <t>23/09/2026</t>
   </si>
   <si>
-    <t>RG33120711IN</t>
+    <t>Speed Post</t>
+  </si>
+  <si>
+    <t>RG11803411IN</t>
   </si>
   <si>
     <t>01/10/2026</t>
   </si>
   <si>
-    <t>TCL-AHD-BL-1003</t>
-  </si>
-  <si>
-    <t>Business Loan</t>
-  </si>
-  <si>
-    <t>Pravin D. Solanki</t>
-  </si>
-  <si>
-    <t>+91 98790 12303</t>
-  </si>
-  <si>
-    <t>pravin.solanki@mail.example</t>
-  </si>
-  <si>
-    <t>7, Shreeji Society, Maninagar</t>
-  </si>
-  <si>
-    <t>380008</t>
-  </si>
-  <si>
-    <t>118034</t>
-  </si>
-  <si>
-    <t>3,65,000</t>
-  </si>
-  <si>
-    <t>BARB0MANINA</t>
-  </si>
-  <si>
-    <t>21950100004471</t>
+    <t>TCL-AHD-PL-1004</t>
+  </si>
+  <si>
+    <t>Mitali R. Shah</t>
+  </si>
+  <si>
+    <t>+91 98790 12304</t>
+  </si>
+  <si>
+    <t>mitali.shah@mail.example</t>
+  </si>
+  <si>
+    <t>C-403, Orchid Greens, Bopal</t>
+  </si>
+  <si>
+    <t>380058</t>
+  </si>
+  <si>
+    <t>560921</t>
+  </si>
+  <si>
+    <t>76,400</t>
+  </si>
+  <si>
+    <t>KKBK0002561</t>
+  </si>
+  <si>
+    <t>7612004893</t>
+  </si>
+  <si>
+    <t>09/08/2026</t>
+  </si>
+  <si>
+    <t>PAYMENT STOPPED</t>
+  </si>
+  <si>
+    <t>15/08/2026</t>
+  </si>
+  <si>
+    <t>RG56092111IN</t>
+  </si>
+  <si>
+    <t>23/08/2026</t>
+  </si>
+  <si>
+    <t>TCL-AHD-TL-1005</t>
+  </si>
+  <si>
+    <t>Two Wheeler Loan</t>
+  </si>
+  <si>
+    <t>Rakesh J. Prajapati</t>
+  </si>
+  <si>
+    <t>+91 98790 12305</t>
+  </si>
+  <si>
+    <t>rakesh.prajapati@mail.example</t>
+  </si>
+  <si>
+    <t>33, Shiv Shakti Nagar, Naroda</t>
+  </si>
+  <si>
+    <t>382330</t>
+  </si>
+  <si>
+    <t>009812</t>
+  </si>
+  <si>
+    <t>58,900</t>
+  </si>
+  <si>
+    <t>PUNB0458600</t>
+  </si>
+  <si>
+    <t>4586000100023911</t>
   </si>
   <si>
     <t>16/09/2026</t>
   </si>
   <si>
-    <t>EXCEEDS ARRANGEMENT</t>
-  </si>
-  <si>
     <t>22/09/2026</t>
   </si>
   <si>
-    <t>Speed Post</t>
-  </si>
-  <si>
-    <t>RG11803411IN</t>
+    <t>RG00981211IN</t>
+  </si>
+  <si>
+    <t>RETURNED</t>
   </si>
   <si>
     <t>30/09/2026</t>
   </si>
   <si>
-    <t>TCL-AHD-PL-1004</t>
-  </si>
-  <si>
-    <t>Mitali R. Shah</t>
-  </si>
-  <si>
-    <t>+91 98790 12304</t>
-  </si>
-  <si>
-    <t>mitali.shah@mail.example</t>
-  </si>
-  <si>
-    <t>C-403, Orchid Greens, Bopal</t>
-  </si>
-  <si>
-    <t>380058</t>
-  </si>
-  <si>
-    <t>560921</t>
-  </si>
-  <si>
-    <t>76,400</t>
-  </si>
-  <si>
-    <t>KKBK0002561</t>
-  </si>
-  <si>
-    <t>7612004893</t>
-  </si>
-  <si>
-    <t>19/09/2026</t>
-  </si>
-  <si>
-    <t>PAYMENT STOPPED</t>
-  </si>
-  <si>
-    <t>25/09/2026</t>
-  </si>
-  <si>
-    <t>RG56092111IN</t>
-  </si>
-  <si>
-    <t>03/10/2026</t>
-  </si>
-  <si>
-    <t>TCL-AHD-TL-1005</t>
-  </si>
-  <si>
-    <t>Two Wheeler Loan</t>
-  </si>
-  <si>
-    <t>Rakesh J. Prajapati</t>
-  </si>
-  <si>
-    <t>+91 98790 12305</t>
-  </si>
-  <si>
-    <t>rakesh.prajapati@mail.example</t>
-  </si>
-  <si>
-    <t>33, Shiv Shakti Nagar, Naroda</t>
-  </si>
-  <si>
-    <t>382330</t>
-  </si>
-  <si>
-    <t>009812</t>
-  </si>
-  <si>
-    <t>58,900</t>
-  </si>
-  <si>
-    <t>PUNB0458600</t>
-  </si>
-  <si>
-    <t>4586000100023911</t>
-  </si>
-  <si>
-    <t>15/09/2026</t>
+    <t>Unclaimed</t>
+  </si>
+  <si>
+    <t>TCL-AHD-BL-1006</t>
+  </si>
+  <si>
+    <t>Sarthak Packaging Pvt Ltd</t>
+  </si>
+  <si>
+    <t>COMPANY</t>
+  </si>
+  <si>
+    <t>Nikhil S. Desai</t>
+  </si>
+  <si>
+    <t>+91 98790 12306</t>
+  </si>
+  <si>
+    <t>accounts@sarthakpack.example</t>
+  </si>
+  <si>
+    <t>Plot 41, GIDC Phase 2, Naroda</t>
+  </si>
+  <si>
+    <t>442190</t>
+  </si>
+  <si>
+    <t>5,12,000</t>
+  </si>
+  <si>
+    <t>UTIB0000080</t>
+  </si>
+  <si>
+    <t>917020045512230</t>
   </si>
   <si>
     <t>21/09/2026</t>
   </si>
   <si>
-    <t>RG00981211IN</t>
-  </si>
-  <si>
-    <t>RETURNED</t>
-  </si>
-  <si>
-    <t>29/09/2026</t>
-  </si>
-  <si>
-    <t>Unclaimed</t>
-  </si>
-  <si>
-    <t>TCL-AHD-BL-1006</t>
-  </si>
-  <si>
-    <t>Sarthak Packaging Pvt Ltd</t>
-  </si>
-  <si>
-    <t>COMPANY</t>
-  </si>
-  <si>
-    <t>Nikhil S. Desai</t>
-  </si>
-  <si>
-    <t>+91 98790 12306</t>
-  </si>
-  <si>
-    <t>accounts@sarthakpack.example</t>
-  </si>
-  <si>
-    <t>Plot 41, GIDC Phase 2, Naroda</t>
-  </si>
-  <si>
-    <t>442190</t>
-  </si>
-  <si>
-    <t>5,12,000</t>
-  </si>
-  <si>
-    <t>UTIB0000080</t>
-  </si>
-  <si>
-    <t>917020045512230</t>
+    <t>27/09/2026</t>
+  </si>
+  <si>
+    <t>RG44219011IN</t>
+  </si>
+  <si>
+    <t>05/10/2026</t>
+  </si>
+  <si>
+    <t>TCL-AHD-PL-1007</t>
+  </si>
+  <si>
+    <t>Jayesh M. Rana</t>
+  </si>
+  <si>
+    <t>+91 98790 12307</t>
+  </si>
+  <si>
+    <t>jayesh.rana@mail.example</t>
+  </si>
+  <si>
+    <t>9, Sahjanand Park, Paldi</t>
+  </si>
+  <si>
+    <t>VADODARA</t>
+  </si>
+  <si>
+    <t>380006</t>
+  </si>
+  <si>
+    <t>671455</t>
+  </si>
+  <si>
+    <t>1,33,250</t>
+  </si>
+  <si>
+    <t>CNRB0002627</t>
+  </si>
+  <si>
+    <t>2627101009981</t>
+  </si>
+  <si>
+    <t>RG67145511IN</t>
+  </si>
+  <si>
+    <t>TCL-AHD-PL-1008</t>
+  </si>
+  <si>
+    <t>Kinjal A. Trivedi</t>
+  </si>
+  <si>
+    <t>+91 98790 12308</t>
+  </si>
+  <si>
+    <t>kinjal.trivedi@mail.example</t>
+  </si>
+  <si>
+    <t>A-22, Satyam Tenements, Satellite</t>
+  </si>
+  <si>
+    <t>38001</t>
+  </si>
+  <si>
+    <t>780312</t>
+  </si>
+  <si>
+    <t>64,800</t>
+  </si>
+  <si>
+    <t>ICIC0000317</t>
+  </si>
+  <si>
+    <t>031701509872</t>
+  </si>
+  <si>
+    <t>RG78031211IN</t>
+  </si>
+  <si>
+    <t>TCL-AHD-BL-1009</t>
+  </si>
+  <si>
+    <t>Devang P. Joshi</t>
+  </si>
+  <si>
+    <t>+91 98790 12309</t>
+  </si>
+  <si>
+    <t>devang.joshi@mail.example</t>
+  </si>
+  <si>
+    <t>5, Rajpath Bungalows, Bodakdev</t>
+  </si>
+  <si>
+    <t>380054</t>
+  </si>
+  <si>
+    <t>253660</t>
+  </si>
+  <si>
+    <t>2,14,000</t>
+  </si>
+  <si>
+    <t>50100332918</t>
+  </si>
+  <si>
+    <t>RG25366011IN</t>
+  </si>
+  <si>
+    <t>253661</t>
+  </si>
+  <si>
+    <t>1,20,000</t>
+  </si>
+  <si>
+    <t>TCL-AHD-PL-1010</t>
+  </si>
+  <si>
+    <t>Shree Ganesh Traders</t>
+  </si>
+  <si>
+    <t>+91 98790 12310</t>
+  </si>
+  <si>
+    <t>ganesh.traders@mail.example</t>
+  </si>
+  <si>
+    <t>18, Nilkanth Society, Navrangpura</t>
+  </si>
+  <si>
+    <t>380009</t>
+  </si>
+  <si>
+    <t>904417</t>
+  </si>
+  <si>
+    <t>87,300</t>
+  </si>
+  <si>
+    <t>38291007788</t>
   </si>
   <si>
     <t>20/09/2026</t>
@@ -409,145 +553,10 @@
     <t>26/09/2026</t>
   </si>
   <si>
-    <t>RG44219011IN</t>
+    <t>RG90441711IN</t>
   </si>
   <si>
     <t>04/10/2026</t>
-  </si>
-  <si>
-    <t>TCL-AHD-PL-1007</t>
-  </si>
-  <si>
-    <t>Jayesh M. Rana</t>
-  </si>
-  <si>
-    <t>+91 98790 12307</t>
-  </si>
-  <si>
-    <t>jayesh.rana@mail.example</t>
-  </si>
-  <si>
-    <t>9, Sahjanand Park, Paldi</t>
-  </si>
-  <si>
-    <t>VADODARA</t>
-  </si>
-  <si>
-    <t>380006</t>
-  </si>
-  <si>
-    <t>671455</t>
-  </si>
-  <si>
-    <t>1,33,250</t>
-  </si>
-  <si>
-    <t>CNRB0002627</t>
-  </si>
-  <si>
-    <t>2627101009981</t>
-  </si>
-  <si>
-    <t>RG67145511IN</t>
-  </si>
-  <si>
-    <t>TCL-AHD-PL-1008</t>
-  </si>
-  <si>
-    <t>Kinjal A. Trivedi</t>
-  </si>
-  <si>
-    <t>+91 98790 12308</t>
-  </si>
-  <si>
-    <t>kinjal.trivedi@mail.example</t>
-  </si>
-  <si>
-    <t>A-22, Satyam Tenements, Satellite</t>
-  </si>
-  <si>
-    <t>38001</t>
-  </si>
-  <si>
-    <t>780312</t>
-  </si>
-  <si>
-    <t>64,800</t>
-  </si>
-  <si>
-    <t>ICIC0000317</t>
-  </si>
-  <si>
-    <t>031701509872</t>
-  </si>
-  <si>
-    <t>RG78031211IN</t>
-  </si>
-  <si>
-    <t>TCL-AHD-BL-1009</t>
-  </si>
-  <si>
-    <t>Devang P. Joshi</t>
-  </si>
-  <si>
-    <t>+91 98790 12309</t>
-  </si>
-  <si>
-    <t>devang.joshi@mail.example</t>
-  </si>
-  <si>
-    <t>5, Rajpath Bungalows, Bodakdev</t>
-  </si>
-  <si>
-    <t>380054</t>
-  </si>
-  <si>
-    <t>253660</t>
-  </si>
-  <si>
-    <t>2,14,000</t>
-  </si>
-  <si>
-    <t>50100332918</t>
-  </si>
-  <si>
-    <t>RG25366011IN</t>
-  </si>
-  <si>
-    <t>253661</t>
-  </si>
-  <si>
-    <t>1,20,000</t>
-  </si>
-  <si>
-    <t>TCL-AHD-PL-1010</t>
-  </si>
-  <si>
-    <t>Shree Ganesh Traders</t>
-  </si>
-  <si>
-    <t>+91 98790 12310</t>
-  </si>
-  <si>
-    <t>ganesh.traders@mail.example</t>
-  </si>
-  <si>
-    <t>18, Nilkanth Society, Navrangpura</t>
-  </si>
-  <si>
-    <t>380009</t>
-  </si>
-  <si>
-    <t>904417</t>
-  </si>
-  <si>
-    <t>87,300</t>
-  </si>
-  <si>
-    <t>38291007788</t>
-  </si>
-  <si>
-    <t>RG90441711IN</t>
   </si>
   <si>
     <t>Y</t>
@@ -1948,7 +1957,7 @@
         <v>177</v>
       </c>
       <c r="P11" t="s">
-        <v>97</v>
+        <v>178</v>
       </c>
       <c r="Q11" t="s">
         <v>48</v>
@@ -1957,19 +1966,19 @@
         <v>49</v>
       </c>
       <c r="S11" t="s">
-        <v>99</v>
+        <v>179</v>
       </c>
       <c r="T11" t="s">
         <v>51</v>
       </c>
       <c r="U11" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="V11" t="s">
         <v>53</v>
       </c>
       <c r="W11" t="s">
-        <v>101</v>
+        <v>181</v>
       </c>
       <c r="X11" t="s">
         <v>37</v>
@@ -1978,7 +1987,7 @@
         <v>37</v>
       </c>
       <c r="Z11" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="AA11">
         <v>0</v>
@@ -1989,13 +1998,13 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="C12" t="s">
         <v>103</v>
       </c>
       <c r="D12" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="E12" t="s">
         <v>36</v>
@@ -2004,37 +2013,37 @@
         <v>37</v>
       </c>
       <c r="G12" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="H12" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="I12" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="J12" t="s">
         <v>41</v>
       </c>
       <c r="K12" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="L12" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="M12" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="N12" t="s">
         <v>79</v>
       </c>
       <c r="O12" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="P12" t="s">
         <v>113</v>
       </c>
       <c r="Q12" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="R12" t="s">
         <v>49</v>
@@ -2046,7 +2055,7 @@
         <v>51</v>
       </c>
       <c r="U12" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="V12" t="s">
         <v>53</v>
@@ -2072,46 +2081,46 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>191</v>
+        <v>194</v>
       </c>
       <c r="C13" t="s">
         <v>71</v>
       </c>
       <c r="D13" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="E13" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="F13" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="G13" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="H13" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="I13" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="J13" t="s">
         <v>41</v>
       </c>
       <c r="K13" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="L13" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="M13" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="N13" t="s">
         <v>95</v>
       </c>
       <c r="O13" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="P13" t="s">
         <v>66</v>
@@ -2129,7 +2138,7 @@
         <v>84</v>
       </c>
       <c r="U13" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
       <c r="V13" t="s">
         <v>53</v>

</xml_diff>